<commit_message>
fix: strengthen proposed budget source traceability
</commit_message>
<xml_diff>
--- a/budget-explorer-web/public/audit/budget-number-audit.xlsx
+++ b/budget-explorer-web/public/audit/budget-number-audit.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Number Ledger" sheetId="1" r:id="Rc5fe0f44e9804b7c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R300ef48b951a4279"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Checks" sheetId="3" r:id="R76ed6530ed0643df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Files" sheetId="4" r:id="Rf7edd8344cb6451e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Notes" sheetId="5" r:id="Re3b5cc8c73b64eef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Number Ledger" sheetId="1" r:id="Ra752eb676cd741ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="Re1955b6c38ea462c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Checks" sheetId="3" r:id="R1c75d04196c4466c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Files" sheetId="4" r:id="R2da16a523b7c4fed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Notes" sheetId="5" r:id="R5f07e775c9964eac"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -404,7 +404,7 @@
         <x:color rgb="FF008A45"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -415,7 +415,7 @@
         <x:color rgb="FFC62828"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE8E6"/>
         </x:patternFill>
       </x:fill>
@@ -426,7 +426,7 @@
         <x:color rgb="FF008A45"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -437,7 +437,7 @@
         <x:color rgb="FF008A45"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -448,7 +448,7 @@
         <x:color rgb="FFC62828"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE8E6"/>
         </x:patternFill>
       </x:fill>
@@ -459,7 +459,7 @@
         <x:color rgb="FF008A45"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -57915,7 +57915,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3d9d14dca0304666"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f56b78076bf417f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -57948,7 +57948,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="43" t="str">
-        <x:v>Generated 2026-07-22T20:02:00.660638+00:00. Exact integer checks use a zero-cent tolerance.</x:v>
+        <x:v>Generated 2026-07-28T19:43:21.128806+00:00. Exact integer checks use a zero-cent tolerance.</x:v>
       </x:c>
       <x:c r="B2" s="43"/>
       <x:c r="C2" s="43"/>
@@ -59158,7 +59158,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R94523748db6b45df"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1e8fb2c60e8e495c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -59319,10 +59319,10 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E8" s="88" t="n">
-        <x:v>3107991</x:v>
+        <x:v>3550753</x:v>
       </x:c>
       <x:c r="F8" s="88" t="str">
-        <x:v>17bb735c1b53110ffc56fa103ed41deb27f535d21b47e76d5227908e7e214ab2</x:v>
+        <x:v>c6fceef2d44a6c8a8bf42d57438843c385fdf07c629dd242b549e958891f6bea</x:v>
       </x:c>
       <x:c r="G8" s="88" t="str">
         <x:v>https://www.miamidade.gov/resources/budget/fy-26-27/proposed/budget-in-brief.pdf</x:v>
@@ -59345,10 +59345,10 @@
         <x:v>282</x:v>
       </x:c>
       <x:c r="E9" s="88" t="n">
-        <x:v>17287129</x:v>
+        <x:v>18015275</x:v>
       </x:c>
       <x:c r="F9" s="88" t="str">
-        <x:v>0f566d2cc7b5d5e1d3b298bae707e0e8285baa6c2d083648d2a61770946585bd</x:v>
+        <x:v>e34859e4ea4528dd114d8bb572c92821087102b507eedd7779b1fc35ffcaf515</x:v>
       </x:c>
       <x:c r="G9" s="88" t="str">
         <x:v>https://www.miamidade.gov/resources/budget/fy-26-27/proposed/volume-1-bookmarks.pdf</x:v>
@@ -59364,7 +59364,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf026886413f84618"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re198590f1fcc424d"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>